<commit_message>
Add Phase E MVP frontend for episode analytics testing.
Scaffold a Next.js app with dashboard, episode list, and detail views wired to enriched FastAPI endpoints and CORS for local dev.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
+++ b/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
@@ -6,18 +6,19 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="780" windowWidth="31580" windowHeight="22600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Review Needed" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Corporate Action Audit" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Reconciliation Fix Audit" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Targeted Validation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="2012 Reconciliation Policy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2012 Snapshot Quality" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2012 Reconciliation Audit" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="2012 Reconciliation Summary" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Version Info" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="V5 Hard Recon Audit" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="V5 Validation" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="READ_ME_DYNAMATIC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review Needed" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Corporate Action Audit" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reconciliation Fix Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Targeted Validation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2012 Reconciliation Policy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2012 Snapshot Quality" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2012 Reconciliation Audit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2012 Reconciliation Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Version Info" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="V5 Hard Recon Audit" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="V5 Validation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -962,6 +963,1452 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech mistake-buy rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>On Sheet1, find stock Dynamatic Tech (sort/filter by Stock Name).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>You should see these two extra rows BEFORE the 2016-06-10 Buy +44:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2016-04-04  Buy  +157  price 1700</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2016-05-31  Sell -157  price BLANK (exit price unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>If your open V5 file does not show them, close it WITHOUT saving and open THIS file instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>/Users/yash/Library/CloudStorage/OneDrive-Personal/PMS-Decision-Platform/02_Final_Master/TRANSACTIONS_MASTER_V5_1_DYNAMATIC_MISTAKE_BUY.xlsx</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
+    <col width="21" customWidth="1" min="4" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45.25" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>First Available Snapshot</t>
+        </is>
+      </c>
+      <c r="C1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Mode</t>
+        </is>
+      </c>
+      <c r="D1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Qty</t>
+        </is>
+      </c>
+      <c r="E1" s="54" t="inlineStr">
+        <is>
+          <t>Rounded First Qty</t>
+        </is>
+      </c>
+      <c r="F1" s="54" t="inlineStr">
+        <is>
+          <t>Master Qty at First Snapshot</t>
+        </is>
+      </c>
+      <c r="G1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Difference</t>
+        </is>
+      </c>
+      <c r="H1" s="54" t="inlineStr">
+        <is>
+          <t>Max Soft-Window Difference</t>
+        </is>
+      </c>
+      <c r="I1" s="54" t="inlineStr">
+        <is>
+          <t>27-Aug Snapshot Qty</t>
+        </is>
+      </c>
+      <c r="J1" s="54" t="inlineStr">
+        <is>
+          <t>Master Qty at 27-Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="54" t="inlineStr">
+        <is>
+          <t>Post-Cutoff Hard Failures</t>
+        </is>
+      </c>
+      <c r="L1" s="54" t="inlineStr">
+        <is>
+          <t>Master Transaction Changes</t>
+        </is>
+      </c>
+      <c r="M1" s="54" t="inlineStr">
+        <is>
+          <t>Final Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="56" t="inlineStr">
+        <is>
+          <t>Amara Raja</t>
+        </is>
+      </c>
+      <c r="B2" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C2" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D2" s="57" t="n">
+        <v>490.1960784313725</v>
+      </c>
+      <c r="E2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="F2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="G2" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="57" t="n">
+        <v>167.4193548387097</v>
+      </c>
+      <c r="I2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="J2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="K2" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M2" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="56" t="inlineStr">
+        <is>
+          <t>Ashiana</t>
+        </is>
+      </c>
+      <c r="B3" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C3" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D3" s="57" t="n">
+        <v>510.948905109489</v>
+      </c>
+      <c r="E3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="F3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="G3" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="57" t="n">
+        <v>117.7415730337079</v>
+      </c>
+      <c r="I3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="J3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="K3" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M3" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="56" t="inlineStr">
+        <is>
+          <t>BharatForg</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C4" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="n">
+        <v>595.2380952380952</v>
+      </c>
+      <c r="E4" s="57" t="n">
+        <v>595</v>
+      </c>
+      <c r="F4" s="57" t="n">
+        <v>595</v>
+      </c>
+      <c r="G4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="57" t="n">
+        <v>127.7102803738318</v>
+      </c>
+      <c r="I4" s="57" t="n">
+        <v>397</v>
+      </c>
+      <c r="J4" s="57" t="n">
+        <v>397</v>
+      </c>
+      <c r="K4" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M4" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="56" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="n">
+        <v>40956</v>
+      </c>
+      <c r="C5" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D5" s="57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G5" s="57" t="n">
+        <v>-250</v>
+      </c>
+      <c r="H5" s="57" t="n">
+        <v>574.3243243243244</v>
+      </c>
+      <c r="I5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="J5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="K5" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M5" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="56" t="inlineStr">
+        <is>
+          <t>Havells</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C6" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="n">
+        <v>389.6103896103896</v>
+      </c>
+      <c r="E6" s="57" t="n">
+        <v>390</v>
+      </c>
+      <c r="F6" s="57" t="n">
+        <v>390</v>
+      </c>
+      <c r="G6" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="57" t="n">
+        <v>130.9326424870466</v>
+      </c>
+      <c r="I6" s="57" t="n">
+        <v>260</v>
+      </c>
+      <c r="J6" s="57" t="n">
+        <v>260</v>
+      </c>
+      <c r="K6" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M6" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="56" t="inlineStr">
+        <is>
+          <t>Kaveri</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C7" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D7" s="57" t="n">
+        <v>156.25</v>
+      </c>
+      <c r="E7" s="57" t="n">
+        <v>156</v>
+      </c>
+      <c r="F7" s="57" t="n">
+        <v>156</v>
+      </c>
+      <c r="G7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="57" t="n">
+        <v>60.50204638472033</v>
+      </c>
+      <c r="I7" s="57" t="n">
+        <v>111</v>
+      </c>
+      <c r="J7" s="57" t="n">
+        <v>111</v>
+      </c>
+      <c r="K7" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M7" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t>NIITTech</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="n">
+        <v>41008</v>
+      </c>
+      <c r="C8" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>371.7472118959108</v>
+      </c>
+      <c r="E8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="F8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="G8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="57" t="n">
+        <v>175.1496062992126</v>
+      </c>
+      <c r="I8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="J8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="K8" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M8" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t>RSSoftware</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="n">
+        <v>41008</v>
+      </c>
+      <c r="C9" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D9" s="57" t="n">
+        <v>781.25</v>
+      </c>
+      <c r="E9" s="57" t="n">
+        <v>781</v>
+      </c>
+      <c r="F9" s="57" t="n">
+        <v>781</v>
+      </c>
+      <c r="G9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="57" t="n">
+        <v>514.4876033057851</v>
+      </c>
+      <c r="I9" s="57" t="n">
+        <v>1093</v>
+      </c>
+      <c r="J9" s="57" t="n">
+        <v>1093</v>
+      </c>
+      <c r="K9" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M9" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>SanghviMov</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C10" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>919.5402298850574</v>
+      </c>
+      <c r="E10" s="57" t="n">
+        <v>920</v>
+      </c>
+      <c r="F10" s="57" t="n">
+        <v>920</v>
+      </c>
+      <c r="G10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="57" t="n">
+        <v>205.7142857142857</v>
+      </c>
+      <c r="I10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M10" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>Technofab</t>
+        </is>
+      </c>
+      <c r="B11" s="55" t="n">
+        <v>41092</v>
+      </c>
+      <c r="C11" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D11" s="57" t="n">
+        <v>367.6470588235294</v>
+      </c>
+      <c r="E11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="F11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="G11" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="57" t="n">
+        <v>22.625</v>
+      </c>
+      <c r="I11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="J11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="K11" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M11" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C12" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="n">
+        <v>387.0967741935484</v>
+      </c>
+      <c r="E12" s="57" t="n">
+        <v>387</v>
+      </c>
+      <c r="F12" s="57" t="n">
+        <v>387</v>
+      </c>
+      <c r="G12" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="57" t="n">
+        <v>348.3809523809524</v>
+      </c>
+      <c r="I12" s="57" t="n">
+        <v>646</v>
+      </c>
+      <c r="J12" s="57" t="n">
+        <v>646</v>
+      </c>
+      <c r="K12" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M12" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t>Zensar</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="n">
+        <v>41023</v>
+      </c>
+      <c r="C13" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D13" s="57" t="n">
+        <v>225.2252252252252</v>
+      </c>
+      <c r="E13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="F13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="G13" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="57" t="n">
+        <v>38.43283582089552</v>
+      </c>
+      <c r="I13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="J13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="K13" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M13" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J2:K13">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>J2=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="84" t="inlineStr">
+        <is>
+          <t>TRANSACTION MASTER VERSION</t>
+        </is>
+      </c>
+      <c r="B1" s="84" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="85" t="inlineStr">
+        <is>
+          <t>Filename</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>TRANSACTIONS_MASTER_V5_HARD_RECON_FIXES.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="85" t="inlineStr">
+        <is>
+          <t>Based on</t>
+        </is>
+      </c>
+      <c r="B3" s="44" t="inlineStr">
+        <is>
+          <t>V4 final with 2012 reconciliation policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="85" t="inlineStr">
+        <is>
+          <t>V5 changes</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>Applied Geometric/Vguard staged sells, Dynamatic missing buy/exit, E2E and Strides date corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="85" t="inlineStr">
+        <is>
+          <t>Unresolved priced item</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech 31-May-2016 exit price/proceeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="85" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="B6" s="61" t="n">
+        <v>46217.46326298611</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="60" t="n"/>
+      <c r="B7" s="61" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="2"/>
+    <col width="40" customWidth="1" min="3" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="82" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="82" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="C1" s="82" t="inlineStr">
+        <is>
+          <t>Old</t>
+        </is>
+      </c>
+      <c r="D1" s="82" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E1" s="82" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="F1" s="82" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B2" s="52" t="inlineStr">
+        <is>
+          <t>Staged sells</t>
+        </is>
+      </c>
+      <c r="C2" s="52" t="inlineStr">
+        <is>
+          <t>16-May-2013 Sell -394; 27-Nov-2013 Sell -181</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>11-May -98; 16-May -296; 31-Oct -8; 27-Nov -173</t>
+        </is>
+      </c>
+      <c r="E2" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot ladders 646 → 548 → 252 and 181 → 173 → 0</t>
+        </is>
+      </c>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="52" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>Staged sell</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>06-May-2013 Sell -625</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>02-May-2013 Sell -295; 06-May-2013 Sell -330</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot ladder 625 → 330 → 0</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Strides</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Date correction</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>2017-09-17 Sell -267</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>12-Sep-2017 Sell -267</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>12Sep17 snapshot shows zero</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Missing buy and inferred exit</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>No pre-Jun-2016 rows</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>04-Apr-2016 Buy +157 @1700; 31-May-2016 Sell -157 with price blank</t>
+        </is>
+      </c>
+      <c r="E5" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot 157 → 0 before separate 10-Jun-2016 Buy +44</t>
+        </is>
+      </c>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>Applied; exit price unresolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="inlineStr">
+        <is>
+          <t>Date correction</t>
+        </is>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-06 Split +9,585</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>05-Jun-2026 Split +9,585</t>
+        </is>
+      </c>
+      <c r="E6" s="52" t="inlineStr">
+        <is>
+          <t>Existing source note points to 05Jun26</t>
+        </is>
+      </c>
+      <c r="F6" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F6">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>ISNUMBER(SEARCH("Applied",F2))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="86" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="86" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="86" t="inlineStr">
+        <is>
+          <t>Expected Qty</t>
+        </is>
+      </c>
+      <c r="D1" s="86" t="inlineStr">
+        <is>
+          <t>Reconstructed Qty</t>
+        </is>
+      </c>
+      <c r="E1" s="86" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="F1" s="86" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B2" s="43" t="n">
+        <v>41394</v>
+      </c>
+      <c r="C2" s="49" t="n">
+        <v>625</v>
+      </c>
+      <c r="D2" s="49" t="n">
+        <v>625</v>
+      </c>
+      <c r="E2" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="n">
+        <v>41396</v>
+      </c>
+      <c r="C3" s="49" t="n">
+        <v>330</v>
+      </c>
+      <c r="D3" s="49" t="n">
+        <v>330</v>
+      </c>
+      <c r="E3" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B4" s="43" t="n">
+        <v>41400</v>
+      </c>
+      <c r="C4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="n">
+        <v>41405</v>
+      </c>
+      <c r="C5" s="49" t="n">
+        <v>548</v>
+      </c>
+      <c r="D5" s="49" t="n">
+        <v>548</v>
+      </c>
+      <c r="E5" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>41410</v>
+      </c>
+      <c r="C6" s="49" t="n">
+        <v>252</v>
+      </c>
+      <c r="D6" s="49" t="n">
+        <v>252</v>
+      </c>
+      <c r="E6" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="n">
+        <v>41570</v>
+      </c>
+      <c r="C7" s="49" t="n">
+        <v>181</v>
+      </c>
+      <c r="D7" s="49" t="n">
+        <v>181</v>
+      </c>
+      <c r="E7" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="n">
+        <v>41578</v>
+      </c>
+      <c r="C8" s="49" t="n">
+        <v>173</v>
+      </c>
+      <c r="D8" s="49" t="n">
+        <v>173</v>
+      </c>
+      <c r="E8" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="n">
+        <v>41605</v>
+      </c>
+      <c r="C9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="n">
+        <v>42464</v>
+      </c>
+      <c r="C10" s="49" t="n">
+        <v>157</v>
+      </c>
+      <c r="D10" s="49" t="n">
+        <v>157</v>
+      </c>
+      <c r="E10" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="n">
+        <v>42521</v>
+      </c>
+      <c r="C11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="n">
+        <v>42531</v>
+      </c>
+      <c r="C12" s="49" t="n">
+        <v>44</v>
+      </c>
+      <c r="D12" s="49" t="n">
+        <v>44</v>
+      </c>
+      <c r="E12" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C13" s="49" t="n">
+        <v>10650</v>
+      </c>
+      <c r="D13" s="49" t="n">
+        <v>10650</v>
+      </c>
+      <c r="E13" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C14" s="49" t="n">
+        <v>7556</v>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>7556</v>
+      </c>
+      <c r="E14" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Strides</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="n">
+        <v>42990</v>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F15">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>F2="PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N526"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
@@ -6666,7 +8113,7 @@
       </c>
       <c r="H198" s="68" t="inlineStr">
         <is>
-          <t>Mistake buy: Portfolio_2016.xlsx / 04Apr16 shows Dynamatic Tech 157 @1700. Bought in error and exited quickly. Kept for quantity continuity / hard reconciliation.</t>
+          <t>LOOK HERE — Mistake buy: Portfolio_2016 04Apr16 Dynamatic Tech 157 @1700. Bought in error, sold quickly. Kept for quantity recon.</t>
         </is>
       </c>
       <c r="I198" s="64" t="inlineStr">
@@ -6695,7 +8142,7 @@
       <c r="G199" s="26" t="n"/>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>Mistake-buy exit: Portfolio_2016.xlsx — Dynamatic Tech absent on 31May16 (qty to 0). Exit trade PRICE NOT AVAILABLE anymore — intentionally blank. Do not invent a price. Quantity -157 retained for hard reconciliation only.</t>
+          <t>LOOK HERE — Mistake-buy EXIT: absent on 31May16. PRICE UNKNOWN — intentionally blank. Qty -157 for recon only.</t>
         </is>
       </c>
       <c r="I199" s="10" t="n"/>
@@ -15814,709 +17261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="84" t="inlineStr">
-        <is>
-          <t>TRANSACTION MASTER VERSION</t>
-        </is>
-      </c>
-      <c r="B1" s="84" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="85" t="inlineStr">
-        <is>
-          <t>Filename</t>
-        </is>
-      </c>
-      <c r="B2" s="44" t="inlineStr">
-        <is>
-          <t>TRANSACTIONS_MASTER_V5_HARD_RECON_FIXES.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="85" t="inlineStr">
-        <is>
-          <t>Based on</t>
-        </is>
-      </c>
-      <c r="B3" s="44" t="inlineStr">
-        <is>
-          <t>V4 final with 2012 reconciliation policy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="85" t="inlineStr">
-        <is>
-          <t>V5 changes</t>
-        </is>
-      </c>
-      <c r="B4" s="44" t="inlineStr">
-        <is>
-          <t>Applied Geometric/Vguard staged sells, Dynamatic missing buy/exit, E2E and Strides date corrections</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="85" t="inlineStr">
-        <is>
-          <t>Unresolved priced item</t>
-        </is>
-      </c>
-      <c r="B5" s="44" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech 31-May-2016 exit price/proceeds</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="85" t="inlineStr">
-        <is>
-          <t>Created</t>
-        </is>
-      </c>
-      <c r="B6" s="61" t="n">
-        <v>46217.46326298611</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="60" t="n"/>
-      <c r="B7" s="61" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="2"/>
-    <col width="40" customWidth="1" min="3" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="82" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="82" t="inlineStr">
-        <is>
-          <t>Change Type</t>
-        </is>
-      </c>
-      <c r="C1" s="82" t="inlineStr">
-        <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="D1" s="82" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E1" s="82" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="F1" s="82" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B2" s="52" t="inlineStr">
-        <is>
-          <t>Staged sells</t>
-        </is>
-      </c>
-      <c r="C2" s="52" t="inlineStr">
-        <is>
-          <t>16-May-2013 Sell -394; 27-Nov-2013 Sell -181</t>
-        </is>
-      </c>
-      <c r="D2" s="52" t="inlineStr">
-        <is>
-          <t>11-May -98; 16-May -296; 31-Oct -8; 27-Nov -173</t>
-        </is>
-      </c>
-      <c r="E2" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot ladders 646 → 548 → 252 and 181 → 173 → 0</t>
-        </is>
-      </c>
-      <c r="F2" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="52" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B3" s="52" t="inlineStr">
-        <is>
-          <t>Staged sell</t>
-        </is>
-      </c>
-      <c r="C3" s="52" t="inlineStr">
-        <is>
-          <t>06-May-2013 Sell -625</t>
-        </is>
-      </c>
-      <c r="D3" s="52" t="inlineStr">
-        <is>
-          <t>02-May-2013 Sell -295; 06-May-2013 Sell -330</t>
-        </is>
-      </c>
-      <c r="E3" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot ladder 625 → 330 → 0</t>
-        </is>
-      </c>
-      <c r="F3" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="52" t="inlineStr">
-        <is>
-          <t>Strides</t>
-        </is>
-      </c>
-      <c r="B4" s="52" t="inlineStr">
-        <is>
-          <t>Date correction</t>
-        </is>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
-        <is>
-          <t>2017-09-17 Sell -267</t>
-        </is>
-      </c>
-      <c r="D4" s="52" t="inlineStr">
-        <is>
-          <t>12-Sep-2017 Sell -267</t>
-        </is>
-      </c>
-      <c r="E4" s="52" t="inlineStr">
-        <is>
-          <t>12Sep17 snapshot shows zero</t>
-        </is>
-      </c>
-      <c r="F4" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="52" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>Missing buy and inferred exit</t>
-        </is>
-      </c>
-      <c r="C5" s="52" t="inlineStr">
-        <is>
-          <t>No pre-Jun-2016 rows</t>
-        </is>
-      </c>
-      <c r="D5" s="52" t="inlineStr">
-        <is>
-          <t>04-Apr-2016 Buy +157 @1700; 31-May-2016 Sell -157 with price blank</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot 157 → 0 before separate 10-Jun-2016 Buy +44</t>
-        </is>
-      </c>
-      <c r="F5" s="52" t="inlineStr">
-        <is>
-          <t>Applied; exit price unresolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="52" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="inlineStr">
-        <is>
-          <t>Date correction</t>
-        </is>
-      </c>
-      <c r="C6" s="52" t="inlineStr">
-        <is>
-          <t>2026-05-06 Split +9,585</t>
-        </is>
-      </c>
-      <c r="D6" s="52" t="inlineStr">
-        <is>
-          <t>05-Jun-2026 Split +9,585</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="inlineStr">
-        <is>
-          <t>Existing source note points to 05Jun26</t>
-        </is>
-      </c>
-      <c r="F6" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="F2:F6">
-    <cfRule type="expression" priority="1" dxfId="1">
-      <formula>ISNUMBER(SEARCH("Applied",F2))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="86" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="86" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="86" t="inlineStr">
-        <is>
-          <t>Expected Qty</t>
-        </is>
-      </c>
-      <c r="D1" s="86" t="inlineStr">
-        <is>
-          <t>Reconstructed Qty</t>
-        </is>
-      </c>
-      <c r="E1" s="86" t="inlineStr">
-        <is>
-          <t>Difference</t>
-        </is>
-      </c>
-      <c r="F1" s="86" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B2" s="43" t="n">
-        <v>41394</v>
-      </c>
-      <c r="C2" s="49" t="n">
-        <v>625</v>
-      </c>
-      <c r="D2" s="49" t="n">
-        <v>625</v>
-      </c>
-      <c r="E2" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B3" s="43" t="n">
-        <v>41396</v>
-      </c>
-      <c r="C3" s="49" t="n">
-        <v>330</v>
-      </c>
-      <c r="D3" s="49" t="n">
-        <v>330</v>
-      </c>
-      <c r="E3" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B4" s="43" t="n">
-        <v>41400</v>
-      </c>
-      <c r="C4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B5" s="43" t="n">
-        <v>41405</v>
-      </c>
-      <c r="C5" s="49" t="n">
-        <v>548</v>
-      </c>
-      <c r="D5" s="49" t="n">
-        <v>548</v>
-      </c>
-      <c r="E5" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B6" s="43" t="n">
-        <v>41410</v>
-      </c>
-      <c r="C6" s="49" t="n">
-        <v>252</v>
-      </c>
-      <c r="D6" s="49" t="n">
-        <v>252</v>
-      </c>
-      <c r="E6" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B7" s="43" t="n">
-        <v>41570</v>
-      </c>
-      <c r="C7" s="49" t="n">
-        <v>181</v>
-      </c>
-      <c r="D7" s="49" t="n">
-        <v>181</v>
-      </c>
-      <c r="E7" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B8" s="43" t="n">
-        <v>41578</v>
-      </c>
-      <c r="C8" s="49" t="n">
-        <v>173</v>
-      </c>
-      <c r="D8" s="49" t="n">
-        <v>173</v>
-      </c>
-      <c r="E8" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B9" s="43" t="n">
-        <v>41605</v>
-      </c>
-      <c r="C9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B10" s="43" t="n">
-        <v>42464</v>
-      </c>
-      <c r="C10" s="49" t="n">
-        <v>157</v>
-      </c>
-      <c r="D10" s="49" t="n">
-        <v>157</v>
-      </c>
-      <c r="E10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B11" s="43" t="n">
-        <v>42521</v>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B12" s="43" t="n">
-        <v>42531</v>
-      </c>
-      <c r="C12" s="49" t="n">
-        <v>44</v>
-      </c>
-      <c r="D12" s="49" t="n">
-        <v>44</v>
-      </c>
-      <c r="E12" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B13" s="43" t="n">
-        <v>46178</v>
-      </c>
-      <c r="C13" s="49" t="n">
-        <v>10650</v>
-      </c>
-      <c r="D13" s="49" t="n">
-        <v>10650</v>
-      </c>
-      <c r="E13" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="n">
-        <v>46195</v>
-      </c>
-      <c r="C14" s="49" t="n">
-        <v>7556</v>
-      </c>
-      <c r="D14" s="49" t="n">
-        <v>7556</v>
-      </c>
-      <c r="E14" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Strides</t>
-        </is>
-      </c>
-      <c r="B15" s="43" t="n">
-        <v>42990</v>
-      </c>
-      <c r="C15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="F2:F15">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>F2="PASS"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17049,7 +17794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17637,7 +18382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18073,7 +18818,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18877,7 +19622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19069,7 +19814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19873,7 +20618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31043,685 +31788,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="3"/>
-    <col width="21" customWidth="1" min="4" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="58" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="45.25" customHeight="1">
-      <c r="A1" s="54" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="54" t="inlineStr">
-        <is>
-          <t>First Available Snapshot</t>
-        </is>
-      </c>
-      <c r="C1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Mode</t>
-        </is>
-      </c>
-      <c r="D1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Qty</t>
-        </is>
-      </c>
-      <c r="E1" s="54" t="inlineStr">
-        <is>
-          <t>Rounded First Qty</t>
-        </is>
-      </c>
-      <c r="F1" s="54" t="inlineStr">
-        <is>
-          <t>Master Qty at First Snapshot</t>
-        </is>
-      </c>
-      <c r="G1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Difference</t>
-        </is>
-      </c>
-      <c r="H1" s="54" t="inlineStr">
-        <is>
-          <t>Max Soft-Window Difference</t>
-        </is>
-      </c>
-      <c r="I1" s="54" t="inlineStr">
-        <is>
-          <t>27-Aug Snapshot Qty</t>
-        </is>
-      </c>
-      <c r="J1" s="54" t="inlineStr">
-        <is>
-          <t>Master Qty at 27-Aug</t>
-        </is>
-      </c>
-      <c r="K1" s="54" t="inlineStr">
-        <is>
-          <t>Post-Cutoff Hard Failures</t>
-        </is>
-      </c>
-      <c r="L1" s="54" t="inlineStr">
-        <is>
-          <t>Master Transaction Changes</t>
-        </is>
-      </c>
-      <c r="M1" s="54" t="inlineStr">
-        <is>
-          <t>Final Treatment</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="56" t="inlineStr">
-        <is>
-          <t>Amara Raja</t>
-        </is>
-      </c>
-      <c r="B2" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C2" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D2" s="57" t="n">
-        <v>490.1960784313725</v>
-      </c>
-      <c r="E2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="F2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="G2" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="57" t="n">
-        <v>167.4193548387097</v>
-      </c>
-      <c r="I2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="J2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="K2" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M2" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="56" t="inlineStr">
-        <is>
-          <t>Ashiana</t>
-        </is>
-      </c>
-      <c r="B3" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C3" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D3" s="57" t="n">
-        <v>510.948905109489</v>
-      </c>
-      <c r="E3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="F3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="G3" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="57" t="n">
-        <v>117.7415730337079</v>
-      </c>
-      <c r="I3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="J3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="K3" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M3" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="56" t="inlineStr">
-        <is>
-          <t>BharatForg</t>
-        </is>
-      </c>
-      <c r="B4" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C4" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D4" s="57" t="n">
-        <v>595.2380952380952</v>
-      </c>
-      <c r="E4" s="57" t="n">
-        <v>595</v>
-      </c>
-      <c r="F4" s="57" t="n">
-        <v>595</v>
-      </c>
-      <c r="G4" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="57" t="n">
-        <v>127.7102803738318</v>
-      </c>
-      <c r="I4" s="57" t="n">
-        <v>397</v>
-      </c>
-      <c r="J4" s="57" t="n">
-        <v>397</v>
-      </c>
-      <c r="K4" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M4" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B5" s="55" t="n">
-        <v>40956</v>
-      </c>
-      <c r="C5" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D5" s="57" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E5" s="57" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G5" s="57" t="n">
-        <v>-250</v>
-      </c>
-      <c r="H5" s="57" t="n">
-        <v>574.3243243243244</v>
-      </c>
-      <c r="I5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="J5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="K5" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M5" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="56" t="inlineStr">
-        <is>
-          <t>Havells</t>
-        </is>
-      </c>
-      <c r="B6" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C6" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D6" s="57" t="n">
-        <v>389.6103896103896</v>
-      </c>
-      <c r="E6" s="57" t="n">
-        <v>390</v>
-      </c>
-      <c r="F6" s="57" t="n">
-        <v>390</v>
-      </c>
-      <c r="G6" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="57" t="n">
-        <v>130.9326424870466</v>
-      </c>
-      <c r="I6" s="57" t="n">
-        <v>260</v>
-      </c>
-      <c r="J6" s="57" t="n">
-        <v>260</v>
-      </c>
-      <c r="K6" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M6" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="56" t="inlineStr">
-        <is>
-          <t>Kaveri</t>
-        </is>
-      </c>
-      <c r="B7" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C7" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D7" s="57" t="n">
-        <v>156.25</v>
-      </c>
-      <c r="E7" s="57" t="n">
-        <v>156</v>
-      </c>
-      <c r="F7" s="57" t="n">
-        <v>156</v>
-      </c>
-      <c r="G7" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="57" t="n">
-        <v>60.50204638472033</v>
-      </c>
-      <c r="I7" s="57" t="n">
-        <v>111</v>
-      </c>
-      <c r="J7" s="57" t="n">
-        <v>111</v>
-      </c>
-      <c r="K7" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M7" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="56" t="inlineStr">
-        <is>
-          <t>NIITTech</t>
-        </is>
-      </c>
-      <c r="B8" s="55" t="n">
-        <v>41008</v>
-      </c>
-      <c r="C8" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D8" s="57" t="n">
-        <v>371.7472118959108</v>
-      </c>
-      <c r="E8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="F8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="G8" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="57" t="n">
-        <v>175.1496062992126</v>
-      </c>
-      <c r="I8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="J8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="K8" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M8" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="56" t="inlineStr">
-        <is>
-          <t>RSSoftware</t>
-        </is>
-      </c>
-      <c r="B9" s="55" t="n">
-        <v>41008</v>
-      </c>
-      <c r="C9" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D9" s="57" t="n">
-        <v>781.25</v>
-      </c>
-      <c r="E9" s="57" t="n">
-        <v>781</v>
-      </c>
-      <c r="F9" s="57" t="n">
-        <v>781</v>
-      </c>
-      <c r="G9" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="57" t="n">
-        <v>514.4876033057851</v>
-      </c>
-      <c r="I9" s="57" t="n">
-        <v>1093</v>
-      </c>
-      <c r="J9" s="57" t="n">
-        <v>1093</v>
-      </c>
-      <c r="K9" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M9" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="56" t="inlineStr">
-        <is>
-          <t>SanghviMov</t>
-        </is>
-      </c>
-      <c r="B10" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C10" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D10" s="57" t="n">
-        <v>919.5402298850574</v>
-      </c>
-      <c r="E10" s="57" t="n">
-        <v>920</v>
-      </c>
-      <c r="F10" s="57" t="n">
-        <v>920</v>
-      </c>
-      <c r="G10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="57" t="n">
-        <v>205.7142857142857</v>
-      </c>
-      <c r="I10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M10" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="56" t="inlineStr">
-        <is>
-          <t>Technofab</t>
-        </is>
-      </c>
-      <c r="B11" s="55" t="n">
-        <v>41092</v>
-      </c>
-      <c r="C11" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D11" s="57" t="n">
-        <v>367.6470588235294</v>
-      </c>
-      <c r="E11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="F11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="G11" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="57" t="n">
-        <v>22.625</v>
-      </c>
-      <c r="I11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="J11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="K11" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M11" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="56" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B12" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C12" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D12" s="57" t="n">
-        <v>387.0967741935484</v>
-      </c>
-      <c r="E12" s="57" t="n">
-        <v>387</v>
-      </c>
-      <c r="F12" s="57" t="n">
-        <v>387</v>
-      </c>
-      <c r="G12" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="57" t="n">
-        <v>348.3809523809524</v>
-      </c>
-      <c r="I12" s="57" t="n">
-        <v>646</v>
-      </c>
-      <c r="J12" s="57" t="n">
-        <v>646</v>
-      </c>
-      <c r="K12" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M12" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="56" t="inlineStr">
-        <is>
-          <t>Zensar</t>
-        </is>
-      </c>
-      <c r="B13" s="55" t="n">
-        <v>41023</v>
-      </c>
-      <c r="C13" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D13" s="57" t="n">
-        <v>225.2252252252252</v>
-      </c>
-      <c r="E13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="F13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="G13" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="57" t="n">
-        <v>38.43283582089552</v>
-      </c>
-      <c r="I13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="J13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="K13" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M13" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="J2:K13">
-    <cfRule type="expression" priority="1" dxfId="1">
-      <formula>J2=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Restore raw transaction master after accidental commit.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
+++ b/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
@@ -6,19 +6,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="780" windowWidth="31580" windowHeight="22600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="READ_ME_DYNAMATIC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Review Needed" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Corporate Action Audit" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reconciliation Fix Audit" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Targeted Validation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2012 Reconciliation Policy" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2012 Snapshot Quality" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="2012 Reconciliation Audit" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="2012 Reconciliation Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Version Info" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="V5 Hard Recon Audit" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="V5 Validation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Review Needed" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Corporate Action Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Reconciliation Fix Audit" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Targeted Validation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2012 Reconciliation Policy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2012 Snapshot Quality" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2012 Reconciliation Audit" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2012 Reconciliation Summary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Version Info" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="V5 Hard Recon Audit" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="V5 Validation" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -963,1452 +962,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech mistake-buy rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>On Sheet1, find stock Dynamatic Tech (sort/filter by Stock Name).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>You should see these two extra rows BEFORE the 2016-06-10 Buy +44:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2016-04-04  Buy  +157  price 1700</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2016-05-31  Sell -157  price BLANK (exit price unknown)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>If your open V5 file does not show them, close it WITHOUT saving and open THIS file instead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>/Users/yash/Library/CloudStorage/OneDrive-Personal/PMS-Decision-Platform/02_Final_Master/TRANSACTIONS_MASTER_V5_1_DYNAMATIC_MISTAKE_BUY.xlsx</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="3"/>
-    <col width="21" customWidth="1" min="4" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="58" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="45.25" customHeight="1">
-      <c r="A1" s="54" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="54" t="inlineStr">
-        <is>
-          <t>First Available Snapshot</t>
-        </is>
-      </c>
-      <c r="C1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Mode</t>
-        </is>
-      </c>
-      <c r="D1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Qty</t>
-        </is>
-      </c>
-      <c r="E1" s="54" t="inlineStr">
-        <is>
-          <t>Rounded First Qty</t>
-        </is>
-      </c>
-      <c r="F1" s="54" t="inlineStr">
-        <is>
-          <t>Master Qty at First Snapshot</t>
-        </is>
-      </c>
-      <c r="G1" s="54" t="inlineStr">
-        <is>
-          <t>First Snapshot Difference</t>
-        </is>
-      </c>
-      <c r="H1" s="54" t="inlineStr">
-        <is>
-          <t>Max Soft-Window Difference</t>
-        </is>
-      </c>
-      <c r="I1" s="54" t="inlineStr">
-        <is>
-          <t>27-Aug Snapshot Qty</t>
-        </is>
-      </c>
-      <c r="J1" s="54" t="inlineStr">
-        <is>
-          <t>Master Qty at 27-Aug</t>
-        </is>
-      </c>
-      <c r="K1" s="54" t="inlineStr">
-        <is>
-          <t>Post-Cutoff Hard Failures</t>
-        </is>
-      </c>
-      <c r="L1" s="54" t="inlineStr">
-        <is>
-          <t>Master Transaction Changes</t>
-        </is>
-      </c>
-      <c r="M1" s="54" t="inlineStr">
-        <is>
-          <t>Final Treatment</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="56" t="inlineStr">
-        <is>
-          <t>Amara Raja</t>
-        </is>
-      </c>
-      <c r="B2" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C2" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D2" s="57" t="n">
-        <v>490.1960784313725</v>
-      </c>
-      <c r="E2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="F2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="G2" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="57" t="n">
-        <v>167.4193548387097</v>
-      </c>
-      <c r="I2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="J2" s="57" t="n">
-        <v>490</v>
-      </c>
-      <c r="K2" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M2" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="56" t="inlineStr">
-        <is>
-          <t>Ashiana</t>
-        </is>
-      </c>
-      <c r="B3" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C3" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D3" s="57" t="n">
-        <v>510.948905109489</v>
-      </c>
-      <c r="E3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="F3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="G3" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="57" t="n">
-        <v>117.7415730337079</v>
-      </c>
-      <c r="I3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="J3" s="57" t="n">
-        <v>511</v>
-      </c>
-      <c r="K3" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M3" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="56" t="inlineStr">
-        <is>
-          <t>BharatForg</t>
-        </is>
-      </c>
-      <c r="B4" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C4" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D4" s="57" t="n">
-        <v>595.2380952380952</v>
-      </c>
-      <c r="E4" s="57" t="n">
-        <v>595</v>
-      </c>
-      <c r="F4" s="57" t="n">
-        <v>595</v>
-      </c>
-      <c r="G4" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="57" t="n">
-        <v>127.7102803738318</v>
-      </c>
-      <c r="I4" s="57" t="n">
-        <v>397</v>
-      </c>
-      <c r="J4" s="57" t="n">
-        <v>397</v>
-      </c>
-      <c r="K4" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M4" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B5" s="55" t="n">
-        <v>40956</v>
-      </c>
-      <c r="C5" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D5" s="57" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E5" s="57" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G5" s="57" t="n">
-        <v>-250</v>
-      </c>
-      <c r="H5" s="57" t="n">
-        <v>574.3243243243244</v>
-      </c>
-      <c r="I5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="J5" s="57" t="n">
-        <v>1250</v>
-      </c>
-      <c r="K5" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M5" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="56" t="inlineStr">
-        <is>
-          <t>Havells</t>
-        </is>
-      </c>
-      <c r="B6" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C6" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D6" s="57" t="n">
-        <v>389.6103896103896</v>
-      </c>
-      <c r="E6" s="57" t="n">
-        <v>390</v>
-      </c>
-      <c r="F6" s="57" t="n">
-        <v>390</v>
-      </c>
-      <c r="G6" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="57" t="n">
-        <v>130.9326424870466</v>
-      </c>
-      <c r="I6" s="57" t="n">
-        <v>260</v>
-      </c>
-      <c r="J6" s="57" t="n">
-        <v>260</v>
-      </c>
-      <c r="K6" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M6" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="56" t="inlineStr">
-        <is>
-          <t>Kaveri</t>
-        </is>
-      </c>
-      <c r="B7" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C7" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D7" s="57" t="n">
-        <v>156.25</v>
-      </c>
-      <c r="E7" s="57" t="n">
-        <v>156</v>
-      </c>
-      <c r="F7" s="57" t="n">
-        <v>156</v>
-      </c>
-      <c r="G7" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="57" t="n">
-        <v>60.50204638472033</v>
-      </c>
-      <c r="I7" s="57" t="n">
-        <v>111</v>
-      </c>
-      <c r="J7" s="57" t="n">
-        <v>111</v>
-      </c>
-      <c r="K7" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M7" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="56" t="inlineStr">
-        <is>
-          <t>NIITTech</t>
-        </is>
-      </c>
-      <c r="B8" s="55" t="n">
-        <v>41008</v>
-      </c>
-      <c r="C8" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D8" s="57" t="n">
-        <v>371.7472118959108</v>
-      </c>
-      <c r="E8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="F8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="G8" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="57" t="n">
-        <v>175.1496062992126</v>
-      </c>
-      <c r="I8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="J8" s="57" t="n">
-        <v>372</v>
-      </c>
-      <c r="K8" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M8" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="56" t="inlineStr">
-        <is>
-          <t>RSSoftware</t>
-        </is>
-      </c>
-      <c r="B9" s="55" t="n">
-        <v>41008</v>
-      </c>
-      <c r="C9" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D9" s="57" t="n">
-        <v>781.25</v>
-      </c>
-      <c r="E9" s="57" t="n">
-        <v>781</v>
-      </c>
-      <c r="F9" s="57" t="n">
-        <v>781</v>
-      </c>
-      <c r="G9" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="57" t="n">
-        <v>514.4876033057851</v>
-      </c>
-      <c r="I9" s="57" t="n">
-        <v>1093</v>
-      </c>
-      <c r="J9" s="57" t="n">
-        <v>1093</v>
-      </c>
-      <c r="K9" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M9" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="56" t="inlineStr">
-        <is>
-          <t>SanghviMov</t>
-        </is>
-      </c>
-      <c r="B10" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C10" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D10" s="57" t="n">
-        <v>919.5402298850574</v>
-      </c>
-      <c r="E10" s="57" t="n">
-        <v>920</v>
-      </c>
-      <c r="F10" s="57" t="n">
-        <v>920</v>
-      </c>
-      <c r="G10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="57" t="n">
-        <v>205.7142857142857</v>
-      </c>
-      <c r="I10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M10" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="56" t="inlineStr">
-        <is>
-          <t>Technofab</t>
-        </is>
-      </c>
-      <c r="B11" s="55" t="n">
-        <v>41092</v>
-      </c>
-      <c r="C11" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D11" s="57" t="n">
-        <v>367.6470588235294</v>
-      </c>
-      <c r="E11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="F11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="G11" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="57" t="n">
-        <v>22.625</v>
-      </c>
-      <c r="I11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="J11" s="57" t="n">
-        <v>368</v>
-      </c>
-      <c r="K11" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M11" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="56" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B12" s="55" t="n">
-        <v>40909</v>
-      </c>
-      <c r="C12" s="57" t="inlineStr">
-        <is>
-          <t>OPENING</t>
-        </is>
-      </c>
-      <c r="D12" s="57" t="n">
-        <v>387.0967741935484</v>
-      </c>
-      <c r="E12" s="57" t="n">
-        <v>387</v>
-      </c>
-      <c r="F12" s="57" t="n">
-        <v>387</v>
-      </c>
-      <c r="G12" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="57" t="n">
-        <v>348.3809523809524</v>
-      </c>
-      <c r="I12" s="57" t="n">
-        <v>646</v>
-      </c>
-      <c r="J12" s="57" t="n">
-        <v>646</v>
-      </c>
-      <c r="K12" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M12" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="56" t="inlineStr">
-        <is>
-          <t>Zensar</t>
-        </is>
-      </c>
-      <c r="B13" s="55" t="n">
-        <v>41023</v>
-      </c>
-      <c r="C13" s="57" t="inlineStr">
-        <is>
-          <t>SOFT</t>
-        </is>
-      </c>
-      <c r="D13" s="57" t="n">
-        <v>225.2252252252252</v>
-      </c>
-      <c r="E13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="F13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="G13" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="57" t="n">
-        <v>38.43283582089552</v>
-      </c>
-      <c r="I13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="J13" s="57" t="n">
-        <v>225</v>
-      </c>
-      <c r="K13" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="52" t="inlineStr">
-        <is>
-          <t>None under 2012 drift policy</t>
-        </is>
-      </c>
-      <c r="M13" s="52" t="inlineStr">
-        <is>
-          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="J2:K13">
-    <cfRule type="expression" priority="1" dxfId="1">
-      <formula>J2=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="84" t="inlineStr">
-        <is>
-          <t>TRANSACTION MASTER VERSION</t>
-        </is>
-      </c>
-      <c r="B1" s="84" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="85" t="inlineStr">
-        <is>
-          <t>Filename</t>
-        </is>
-      </c>
-      <c r="B2" s="44" t="inlineStr">
-        <is>
-          <t>TRANSACTIONS_MASTER_V5_HARD_RECON_FIXES.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="85" t="inlineStr">
-        <is>
-          <t>Based on</t>
-        </is>
-      </c>
-      <c r="B3" s="44" t="inlineStr">
-        <is>
-          <t>V4 final with 2012 reconciliation policy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="85" t="inlineStr">
-        <is>
-          <t>V5 changes</t>
-        </is>
-      </c>
-      <c r="B4" s="44" t="inlineStr">
-        <is>
-          <t>Applied Geometric/Vguard staged sells, Dynamatic missing buy/exit, E2E and Strides date corrections</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="85" t="inlineStr">
-        <is>
-          <t>Unresolved priced item</t>
-        </is>
-      </c>
-      <c r="B5" s="44" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech 31-May-2016 exit price/proceeds</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="85" t="inlineStr">
-        <is>
-          <t>Created</t>
-        </is>
-      </c>
-      <c r="B6" s="61" t="n">
-        <v>46217.46326298611</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="60" t="n"/>
-      <c r="B7" s="61" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="2"/>
-    <col width="40" customWidth="1" min="3" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="82" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="82" t="inlineStr">
-        <is>
-          <t>Change Type</t>
-        </is>
-      </c>
-      <c r="C1" s="82" t="inlineStr">
-        <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="D1" s="82" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E1" s="82" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="F1" s="82" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B2" s="52" t="inlineStr">
-        <is>
-          <t>Staged sells</t>
-        </is>
-      </c>
-      <c r="C2" s="52" t="inlineStr">
-        <is>
-          <t>16-May-2013 Sell -394; 27-Nov-2013 Sell -181</t>
-        </is>
-      </c>
-      <c r="D2" s="52" t="inlineStr">
-        <is>
-          <t>11-May -98; 16-May -296; 31-Oct -8; 27-Nov -173</t>
-        </is>
-      </c>
-      <c r="E2" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot ladders 646 → 548 → 252 and 181 → 173 → 0</t>
-        </is>
-      </c>
-      <c r="F2" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="52" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B3" s="52" t="inlineStr">
-        <is>
-          <t>Staged sell</t>
-        </is>
-      </c>
-      <c r="C3" s="52" t="inlineStr">
-        <is>
-          <t>06-May-2013 Sell -625</t>
-        </is>
-      </c>
-      <c r="D3" s="52" t="inlineStr">
-        <is>
-          <t>02-May-2013 Sell -295; 06-May-2013 Sell -330</t>
-        </is>
-      </c>
-      <c r="E3" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot ladder 625 → 330 → 0</t>
-        </is>
-      </c>
-      <c r="F3" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="52" t="inlineStr">
-        <is>
-          <t>Strides</t>
-        </is>
-      </c>
-      <c r="B4" s="52" t="inlineStr">
-        <is>
-          <t>Date correction</t>
-        </is>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
-        <is>
-          <t>2017-09-17 Sell -267</t>
-        </is>
-      </c>
-      <c r="D4" s="52" t="inlineStr">
-        <is>
-          <t>12-Sep-2017 Sell -267</t>
-        </is>
-      </c>
-      <c r="E4" s="52" t="inlineStr">
-        <is>
-          <t>12Sep17 snapshot shows zero</t>
-        </is>
-      </c>
-      <c r="F4" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="52" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>Missing buy and inferred exit</t>
-        </is>
-      </c>
-      <c r="C5" s="52" t="inlineStr">
-        <is>
-          <t>No pre-Jun-2016 rows</t>
-        </is>
-      </c>
-      <c r="D5" s="52" t="inlineStr">
-        <is>
-          <t>04-Apr-2016 Buy +157 @1700; 31-May-2016 Sell -157 with price blank</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="inlineStr">
-        <is>
-          <t>Snapshot 157 → 0 before separate 10-Jun-2016 Buy +44</t>
-        </is>
-      </c>
-      <c r="F5" s="52" t="inlineStr">
-        <is>
-          <t>Applied; exit price unresolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="52" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="inlineStr">
-        <is>
-          <t>Date correction</t>
-        </is>
-      </c>
-      <c r="C6" s="52" t="inlineStr">
-        <is>
-          <t>2026-05-06 Split +9,585</t>
-        </is>
-      </c>
-      <c r="D6" s="52" t="inlineStr">
-        <is>
-          <t>05-Jun-2026 Split +9,585</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="inlineStr">
-        <is>
-          <t>Existing source note points to 05Jun26</t>
-        </is>
-      </c>
-      <c r="F6" s="52" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="F2:F6">
-    <cfRule type="expression" priority="1" dxfId="1">
-      <formula>ISNUMBER(SEARCH("Applied",F2))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="86" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B1" s="86" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="86" t="inlineStr">
-        <is>
-          <t>Expected Qty</t>
-        </is>
-      </c>
-      <c r="D1" s="86" t="inlineStr">
-        <is>
-          <t>Reconstructed Qty</t>
-        </is>
-      </c>
-      <c r="E1" s="86" t="inlineStr">
-        <is>
-          <t>Difference</t>
-        </is>
-      </c>
-      <c r="F1" s="86" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B2" s="43" t="n">
-        <v>41394</v>
-      </c>
-      <c r="C2" s="49" t="n">
-        <v>625</v>
-      </c>
-      <c r="D2" s="49" t="n">
-        <v>625</v>
-      </c>
-      <c r="E2" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B3" s="43" t="n">
-        <v>41396</v>
-      </c>
-      <c r="C3" s="49" t="n">
-        <v>330</v>
-      </c>
-      <c r="D3" s="49" t="n">
-        <v>330</v>
-      </c>
-      <c r="E3" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Geometric</t>
-        </is>
-      </c>
-      <c r="B4" s="43" t="n">
-        <v>41400</v>
-      </c>
-      <c r="C4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B5" s="43" t="n">
-        <v>41405</v>
-      </c>
-      <c r="C5" s="49" t="n">
-        <v>548</v>
-      </c>
-      <c r="D5" s="49" t="n">
-        <v>548</v>
-      </c>
-      <c r="E5" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B6" s="43" t="n">
-        <v>41410</v>
-      </c>
-      <c r="C6" s="49" t="n">
-        <v>252</v>
-      </c>
-      <c r="D6" s="49" t="n">
-        <v>252</v>
-      </c>
-      <c r="E6" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B7" s="43" t="n">
-        <v>41570</v>
-      </c>
-      <c r="C7" s="49" t="n">
-        <v>181</v>
-      </c>
-      <c r="D7" s="49" t="n">
-        <v>181</v>
-      </c>
-      <c r="E7" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B8" s="43" t="n">
-        <v>41578</v>
-      </c>
-      <c r="C8" s="49" t="n">
-        <v>173</v>
-      </c>
-      <c r="D8" s="49" t="n">
-        <v>173</v>
-      </c>
-      <c r="E8" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Vguard</t>
-        </is>
-      </c>
-      <c r="B9" s="43" t="n">
-        <v>41605</v>
-      </c>
-      <c r="C9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B10" s="43" t="n">
-        <v>42464</v>
-      </c>
-      <c r="C10" s="49" t="n">
-        <v>157</v>
-      </c>
-      <c r="D10" s="49" t="n">
-        <v>157</v>
-      </c>
-      <c r="E10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B11" s="43" t="n">
-        <v>42521</v>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Dynamatic Tech</t>
-        </is>
-      </c>
-      <c r="B12" s="43" t="n">
-        <v>42531</v>
-      </c>
-      <c r="C12" s="49" t="n">
-        <v>44</v>
-      </c>
-      <c r="D12" s="49" t="n">
-        <v>44</v>
-      </c>
-      <c r="E12" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B13" s="43" t="n">
-        <v>46178</v>
-      </c>
-      <c r="C13" s="49" t="n">
-        <v>10650</v>
-      </c>
-      <c r="D13" s="49" t="n">
-        <v>10650</v>
-      </c>
-      <c r="E13" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E2E</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="n">
-        <v>46195</v>
-      </c>
-      <c r="C14" s="49" t="n">
-        <v>7556</v>
-      </c>
-      <c r="D14" s="49" t="n">
-        <v>7556</v>
-      </c>
-      <c r="E14" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Strides</t>
-        </is>
-      </c>
-      <c r="B15" s="43" t="n">
-        <v>42990</v>
-      </c>
-      <c r="C15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="F2:F15">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>F2="PASS"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:N526"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
@@ -8113,7 +6666,7 @@
       </c>
       <c r="H198" s="68" t="inlineStr">
         <is>
-          <t>LOOK HERE — Mistake buy: Portfolio_2016 04Apr16 Dynamatic Tech 157 @1700. Bought in error, sold quickly. Kept for quantity recon.</t>
+          <t>Mistake buy: Portfolio_2016.xlsx / 04Apr16 shows Dynamatic Tech 157 @1700. Bought in error and exited quickly. Kept for quantity continuity / hard reconciliation.</t>
         </is>
       </c>
       <c r="I198" s="64" t="inlineStr">
@@ -8142,7 +6695,7 @@
       <c r="G199" s="26" t="n"/>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>LOOK HERE — Mistake-buy EXIT: absent on 31May16. PRICE UNKNOWN — intentionally blank. Qty -157 for recon only.</t>
+          <t>Mistake-buy exit: Portfolio_2016.xlsx — Dynamatic Tech absent on 31May16 (qty to 0). Exit trade PRICE NOT AVAILABLE anymore — intentionally blank. Do not invent a price. Quantity -157 retained for hard reconciliation only.</t>
         </is>
       </c>
       <c r="I199" s="10" t="n"/>
@@ -17261,7 +15814,709 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="84" t="inlineStr">
+        <is>
+          <t>TRANSACTION MASTER VERSION</t>
+        </is>
+      </c>
+      <c r="B1" s="84" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="85" t="inlineStr">
+        <is>
+          <t>Filename</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>TRANSACTIONS_MASTER_V5_HARD_RECON_FIXES.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="85" t="inlineStr">
+        <is>
+          <t>Based on</t>
+        </is>
+      </c>
+      <c r="B3" s="44" t="inlineStr">
+        <is>
+          <t>V4 final with 2012 reconciliation policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="85" t="inlineStr">
+        <is>
+          <t>V5 changes</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>Applied Geometric/Vguard staged sells, Dynamatic missing buy/exit, E2E and Strides date corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="85" t="inlineStr">
+        <is>
+          <t>Unresolved priced item</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech 31-May-2016 exit price/proceeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="85" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="B6" s="61" t="n">
+        <v>46217.46326298611</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="60" t="n"/>
+      <c r="B7" s="61" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="2"/>
+    <col width="40" customWidth="1" min="3" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="82" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="82" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="C1" s="82" t="inlineStr">
+        <is>
+          <t>Old</t>
+        </is>
+      </c>
+      <c r="D1" s="82" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="E1" s="82" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="F1" s="82" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B2" s="52" t="inlineStr">
+        <is>
+          <t>Staged sells</t>
+        </is>
+      </c>
+      <c r="C2" s="52" t="inlineStr">
+        <is>
+          <t>16-May-2013 Sell -394; 27-Nov-2013 Sell -181</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>11-May -98; 16-May -296; 31-Oct -8; 27-Nov -173</t>
+        </is>
+      </c>
+      <c r="E2" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot ladders 646 → 548 → 252 and 181 → 173 → 0</t>
+        </is>
+      </c>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="52" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>Staged sell</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>06-May-2013 Sell -625</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>02-May-2013 Sell -295; 06-May-2013 Sell -330</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot ladder 625 → 330 → 0</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Strides</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Date correction</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>2017-09-17 Sell -267</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>12-Sep-2017 Sell -267</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>12Sep17 snapshot shows zero</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Missing buy and inferred exit</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>No pre-Jun-2016 rows</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>04-Apr-2016 Buy +157 @1700; 31-May-2016 Sell -157 with price blank</t>
+        </is>
+      </c>
+      <c r="E5" s="52" t="inlineStr">
+        <is>
+          <t>Snapshot 157 → 0 before separate 10-Jun-2016 Buy +44</t>
+        </is>
+      </c>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>Applied; exit price unresolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="inlineStr">
+        <is>
+          <t>Date correction</t>
+        </is>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-06 Split +9,585</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>05-Jun-2026 Split +9,585</t>
+        </is>
+      </c>
+      <c r="E6" s="52" t="inlineStr">
+        <is>
+          <t>Existing source note points to 05Jun26</t>
+        </is>
+      </c>
+      <c r="F6" s="52" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F6">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>ISNUMBER(SEARCH("Applied",F2))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="86" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="86" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="86" t="inlineStr">
+        <is>
+          <t>Expected Qty</t>
+        </is>
+      </c>
+      <c r="D1" s="86" t="inlineStr">
+        <is>
+          <t>Reconstructed Qty</t>
+        </is>
+      </c>
+      <c r="E1" s="86" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="F1" s="86" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B2" s="43" t="n">
+        <v>41394</v>
+      </c>
+      <c r="C2" s="49" t="n">
+        <v>625</v>
+      </c>
+      <c r="D2" s="49" t="n">
+        <v>625</v>
+      </c>
+      <c r="E2" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="n">
+        <v>41396</v>
+      </c>
+      <c r="C3" s="49" t="n">
+        <v>330</v>
+      </c>
+      <c r="D3" s="49" t="n">
+        <v>330</v>
+      </c>
+      <c r="E3" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B4" s="43" t="n">
+        <v>41400</v>
+      </c>
+      <c r="C4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="n">
+        <v>41405</v>
+      </c>
+      <c r="C5" s="49" t="n">
+        <v>548</v>
+      </c>
+      <c r="D5" s="49" t="n">
+        <v>548</v>
+      </c>
+      <c r="E5" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>41410</v>
+      </c>
+      <c r="C6" s="49" t="n">
+        <v>252</v>
+      </c>
+      <c r="D6" s="49" t="n">
+        <v>252</v>
+      </c>
+      <c r="E6" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="n">
+        <v>41570</v>
+      </c>
+      <c r="C7" s="49" t="n">
+        <v>181</v>
+      </c>
+      <c r="D7" s="49" t="n">
+        <v>181</v>
+      </c>
+      <c r="E7" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="n">
+        <v>41578</v>
+      </c>
+      <c r="C8" s="49" t="n">
+        <v>173</v>
+      </c>
+      <c r="D8" s="49" t="n">
+        <v>173</v>
+      </c>
+      <c r="E8" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="n">
+        <v>41605</v>
+      </c>
+      <c r="C9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="n">
+        <v>42464</v>
+      </c>
+      <c r="C10" s="49" t="n">
+        <v>157</v>
+      </c>
+      <c r="D10" s="49" t="n">
+        <v>157</v>
+      </c>
+      <c r="E10" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="n">
+        <v>42521</v>
+      </c>
+      <c r="C11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dynamatic Tech</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="n">
+        <v>42531</v>
+      </c>
+      <c r="C12" s="49" t="n">
+        <v>44</v>
+      </c>
+      <c r="D12" s="49" t="n">
+        <v>44</v>
+      </c>
+      <c r="E12" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C13" s="49" t="n">
+        <v>10650</v>
+      </c>
+      <c r="D13" s="49" t="n">
+        <v>10650</v>
+      </c>
+      <c r="E13" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C14" s="49" t="n">
+        <v>7556</v>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>7556</v>
+      </c>
+      <c r="E14" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Strides</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="n">
+        <v>42990</v>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F15">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>F2="PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17794,7 +17049,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18382,7 +17637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18818,7 +18073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19622,7 +18877,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19814,7 +19069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20618,7 +19873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31788,4 +31043,685 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
+    <col width="21" customWidth="1" min="4" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45.25" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>First Available Snapshot</t>
+        </is>
+      </c>
+      <c r="C1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Mode</t>
+        </is>
+      </c>
+      <c r="D1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Qty</t>
+        </is>
+      </c>
+      <c r="E1" s="54" t="inlineStr">
+        <is>
+          <t>Rounded First Qty</t>
+        </is>
+      </c>
+      <c r="F1" s="54" t="inlineStr">
+        <is>
+          <t>Master Qty at First Snapshot</t>
+        </is>
+      </c>
+      <c r="G1" s="54" t="inlineStr">
+        <is>
+          <t>First Snapshot Difference</t>
+        </is>
+      </c>
+      <c r="H1" s="54" t="inlineStr">
+        <is>
+          <t>Max Soft-Window Difference</t>
+        </is>
+      </c>
+      <c r="I1" s="54" t="inlineStr">
+        <is>
+          <t>27-Aug Snapshot Qty</t>
+        </is>
+      </c>
+      <c r="J1" s="54" t="inlineStr">
+        <is>
+          <t>Master Qty at 27-Aug</t>
+        </is>
+      </c>
+      <c r="K1" s="54" t="inlineStr">
+        <is>
+          <t>Post-Cutoff Hard Failures</t>
+        </is>
+      </c>
+      <c r="L1" s="54" t="inlineStr">
+        <is>
+          <t>Master Transaction Changes</t>
+        </is>
+      </c>
+      <c r="M1" s="54" t="inlineStr">
+        <is>
+          <t>Final Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="56" t="inlineStr">
+        <is>
+          <t>Amara Raja</t>
+        </is>
+      </c>
+      <c r="B2" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C2" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D2" s="57" t="n">
+        <v>490.1960784313725</v>
+      </c>
+      <c r="E2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="F2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="G2" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="57" t="n">
+        <v>167.4193548387097</v>
+      </c>
+      <c r="I2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="J2" s="57" t="n">
+        <v>490</v>
+      </c>
+      <c r="K2" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M2" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="56" t="inlineStr">
+        <is>
+          <t>Ashiana</t>
+        </is>
+      </c>
+      <c r="B3" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C3" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D3" s="57" t="n">
+        <v>510.948905109489</v>
+      </c>
+      <c r="E3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="F3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="G3" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="57" t="n">
+        <v>117.7415730337079</v>
+      </c>
+      <c r="I3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="J3" s="57" t="n">
+        <v>511</v>
+      </c>
+      <c r="K3" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M3" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="56" t="inlineStr">
+        <is>
+          <t>BharatForg</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C4" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="n">
+        <v>595.2380952380952</v>
+      </c>
+      <c r="E4" s="57" t="n">
+        <v>595</v>
+      </c>
+      <c r="F4" s="57" t="n">
+        <v>595</v>
+      </c>
+      <c r="G4" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="57" t="n">
+        <v>127.7102803738318</v>
+      </c>
+      <c r="I4" s="57" t="n">
+        <v>397</v>
+      </c>
+      <c r="J4" s="57" t="n">
+        <v>397</v>
+      </c>
+      <c r="K4" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M4" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="56" t="inlineStr">
+        <is>
+          <t>Geometric</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="n">
+        <v>40956</v>
+      </c>
+      <c r="C5" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D5" s="57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G5" s="57" t="n">
+        <v>-250</v>
+      </c>
+      <c r="H5" s="57" t="n">
+        <v>574.3243243243244</v>
+      </c>
+      <c r="I5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="J5" s="57" t="n">
+        <v>1250</v>
+      </c>
+      <c r="K5" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M5" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="56" t="inlineStr">
+        <is>
+          <t>Havells</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C6" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="n">
+        <v>389.6103896103896</v>
+      </c>
+      <c r="E6" s="57" t="n">
+        <v>390</v>
+      </c>
+      <c r="F6" s="57" t="n">
+        <v>390</v>
+      </c>
+      <c r="G6" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="57" t="n">
+        <v>130.9326424870466</v>
+      </c>
+      <c r="I6" s="57" t="n">
+        <v>260</v>
+      </c>
+      <c r="J6" s="57" t="n">
+        <v>260</v>
+      </c>
+      <c r="K6" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M6" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="56" t="inlineStr">
+        <is>
+          <t>Kaveri</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C7" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D7" s="57" t="n">
+        <v>156.25</v>
+      </c>
+      <c r="E7" s="57" t="n">
+        <v>156</v>
+      </c>
+      <c r="F7" s="57" t="n">
+        <v>156</v>
+      </c>
+      <c r="G7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="57" t="n">
+        <v>60.50204638472033</v>
+      </c>
+      <c r="I7" s="57" t="n">
+        <v>111</v>
+      </c>
+      <c r="J7" s="57" t="n">
+        <v>111</v>
+      </c>
+      <c r="K7" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M7" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t>NIITTech</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="n">
+        <v>41008</v>
+      </c>
+      <c r="C8" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>371.7472118959108</v>
+      </c>
+      <c r="E8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="F8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="G8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="57" t="n">
+        <v>175.1496062992126</v>
+      </c>
+      <c r="I8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="J8" s="57" t="n">
+        <v>372</v>
+      </c>
+      <c r="K8" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M8" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t>RSSoftware</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="n">
+        <v>41008</v>
+      </c>
+      <c r="C9" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D9" s="57" t="n">
+        <v>781.25</v>
+      </c>
+      <c r="E9" s="57" t="n">
+        <v>781</v>
+      </c>
+      <c r="F9" s="57" t="n">
+        <v>781</v>
+      </c>
+      <c r="G9" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="57" t="n">
+        <v>514.4876033057851</v>
+      </c>
+      <c r="I9" s="57" t="n">
+        <v>1093</v>
+      </c>
+      <c r="J9" s="57" t="n">
+        <v>1093</v>
+      </c>
+      <c r="K9" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M9" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>SanghviMov</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C10" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>919.5402298850574</v>
+      </c>
+      <c r="E10" s="57" t="n">
+        <v>920</v>
+      </c>
+      <c r="F10" s="57" t="n">
+        <v>920</v>
+      </c>
+      <c r="G10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="57" t="n">
+        <v>205.7142857142857</v>
+      </c>
+      <c r="I10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M10" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>Technofab</t>
+        </is>
+      </c>
+      <c r="B11" s="55" t="n">
+        <v>41092</v>
+      </c>
+      <c r="C11" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D11" s="57" t="n">
+        <v>367.6470588235294</v>
+      </c>
+      <c r="E11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="F11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="G11" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="57" t="n">
+        <v>22.625</v>
+      </c>
+      <c r="I11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="J11" s="57" t="n">
+        <v>368</v>
+      </c>
+      <c r="K11" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M11" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Vguard</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>40909</v>
+      </c>
+      <c r="C12" s="57" t="inlineStr">
+        <is>
+          <t>OPENING</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="n">
+        <v>387.0967741935484</v>
+      </c>
+      <c r="E12" s="57" t="n">
+        <v>387</v>
+      </c>
+      <c r="F12" s="57" t="n">
+        <v>387</v>
+      </c>
+      <c r="G12" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="57" t="n">
+        <v>348.3809523809524</v>
+      </c>
+      <c r="I12" s="57" t="n">
+        <v>646</v>
+      </c>
+      <c r="J12" s="57" t="n">
+        <v>646</v>
+      </c>
+      <c r="K12" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M12" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t>Zensar</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="n">
+        <v>41023</v>
+      </c>
+      <c r="C13" s="57" t="inlineStr">
+        <is>
+          <t>SOFT</t>
+        </is>
+      </c>
+      <c r="D13" s="57" t="n">
+        <v>225.2252252252252</v>
+      </c>
+      <c r="E13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="F13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="G13" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="57" t="n">
+        <v>38.43283582089552</v>
+      </c>
+      <c r="I13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="J13" s="57" t="n">
+        <v>225</v>
+      </c>
+      <c r="K13" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="52" t="inlineStr">
+        <is>
+          <t>None under 2012 drift policy</t>
+        </is>
+      </c>
+      <c r="M13" s="52" t="inlineStr">
+        <is>
+          <t>Soft warnings before 27-Aug-2012; hard reconciliation from 27-Aug-2012</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J2:K13">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>J2=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ship holdings UX, nav groups, pivot/client tools, and ponytail cleanup.
Open holdings use first-buy→current return and show portfolio weight; nav is dropdown-grouped; drop dead stubs/deps and share BSE HTTP helpers; include harvest, pivot bhav, and client portfolio flows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
+++ b/data/raw/transactions/MASTER_TRANSACTIONS_V1.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="780" windowWidth="31580" windowHeight="22600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="READ_ME_DYNAMATIC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Review Needed" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Corporate Action Audit" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reconciliation Fix Audit" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Targeted Validation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2012 Reconciliation Policy" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2012 Snapshot Quality" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="2012 Reconciliation Audit" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="2012 Reconciliation Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Version Info" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="V5 Hard Recon Audit" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="V5 Validation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ_ME_DYNAMATIC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Needed" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Action Audit" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation Fix Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeted Validation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2012 Reconciliation Policy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2012 Snapshot Quality" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2012 Reconciliation Audit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2012 Reconciliation Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Info" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5 Hard Recon Audit" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V5 Validation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -27,12 +27,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0;[Red]\(#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="#,##0.00;[Red]\(#,##0.00\);\-"/>
     <numFmt numFmtId="168" formatCode="dd\-mmm\-yyyy\ hh:mm"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -253,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -507,6 +508,7 @@
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2409,7 +2411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N526"/>
+  <dimension ref="A1:N532"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17250,6 +17252,180 @@
       <c r="I526" s="77" t="n"/>
       <c r="J526" s="77" t="n"/>
       <c r="K526" s="77" t="n"/>
+    </row>
+    <row r="527">
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>HEG</t>
+        </is>
+      </c>
+      <c r="C527" s="89" t="n">
+        <v>46227</v>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>562</v>
+      </c>
+      <c r="F527" t="n">
+        <v>643.95</v>
+      </c>
+      <c r="G527" t="n">
+        <v>358036</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 24Jul26: Add 562@643.95 = 358036</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Aurionpro</t>
+        </is>
+      </c>
+      <c r="C528" s="89" t="n">
+        <v>46231</v>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>-604</v>
+      </c>
+      <c r="F528" t="n">
+        <v>745.9299999999999</v>
+      </c>
+      <c r="G528" t="n">
+        <v>450542</v>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 28Jul26: Sell 604@745.93 = 450542</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>AtherEnerg</t>
+        </is>
+      </c>
+      <c r="C529" s="89" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>315</v>
+      </c>
+      <c r="F529" t="n">
+        <v>1451.14</v>
+      </c>
+      <c r="G529" t="n">
+        <v>457109</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 04Aug26: Add 315@1451.14 = 457109</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>WelEnt</t>
+        </is>
+      </c>
+      <c r="C530" s="89" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>-465</v>
+      </c>
+      <c r="F530" t="n">
+        <v>580.92</v>
+      </c>
+      <c r="G530" t="n">
+        <v>270128</v>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 04Aug26: Sell 465@580.92 = 270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>HEG</t>
+        </is>
+      </c>
+      <c r="C531" s="89" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>550</v>
+      </c>
+      <c r="F531" t="n">
+        <v>683.63</v>
+      </c>
+      <c r="G531" t="n">
+        <v>375997</v>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 10Aug26: Add 550@683.63 = 375997</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>WelEnt</t>
+        </is>
+      </c>
+      <c r="C532" s="89" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>-1389</v>
+      </c>
+      <c r="F532" t="n">
+        <v>581.25</v>
+      </c>
+      <c r="G532" t="n">
+        <v>807356</v>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Portfolio_2026.xlsx / 10Aug26: Sell 1389@581.25 = 807356</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D427">

</xml_diff>